<commit_message>
chore: save current workspace state without mp4 files
</commit_message>
<xml_diff>
--- a/02_product/02_course_creation/00_curriculum_and_index/05_web_index.xlsx
+++ b/02_product/02_course_creation/00_curriculum_and_index/05_web_index.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\vault\Koreanwithji_vault\02_product\02_course_creation\00_curriculum_and_index\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BE0C8F2-579A-4D17-9E3B-97AF60F31E73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DDDE4BC-6BB5-4729-B6B0-DDD6218AB763}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{DDE8F56D-E551-4862-8AC9-22257F07E936}"/>
+    <workbookView xWindow="-38520" yWindow="7500" windowWidth="38640" windowHeight="21120" xr2:uid="{DDE8F56D-E551-4862-8AC9-22257F07E936}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="미매핑" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="35">
   <si>
     <t>Ji 레벨</t>
   </si>
@@ -88,9 +88,6 @@
     <t>You in Korean</t>
   </si>
   <si>
-    <t>Reddit</t>
-  </si>
-  <si>
     <t>How to say "you" politely in Korean</t>
   </si>
   <si>
@@ -117,10 +114,6 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>Reddit</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>X</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
@@ -142,13 +135,22 @@
   </si>
   <si>
     <t>05_Reddit</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>링크 및 경로</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>영상 타이틀</t>
+    <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -448,7 +450,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -517,9 +519,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="1" applyFont="1" applyAlignment="1">
@@ -557,9 +556,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="7" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="7" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="7" borderId="7" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -896,22 +892,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19BC9819-3AE3-40CF-B918-34373651DDDD}">
-  <dimension ref="A1:K5"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5"/>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.7"/>
   <cols>
     <col min="1" max="1" width="8.09765625" style="18" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="3.5" style="18" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20" style="18" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.1484375" style="18" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.25" style="18" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9" style="18"/>
-    <col min="7" max="7" width="11.34765625" style="18" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="64.25" style="18" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="116.5" style="18" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="9" style="18"/>
+    <col min="4" max="4" width="9.69921875" style="18" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.75" style="18" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="64.25" style="18" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="116.5" style="18" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9" style="18"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="4" customFormat="1" ht="49.5">
+    <row r="1" spans="1:9" s="4" customFormat="1" ht="49.5" x14ac:dyDescent="0.7">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -924,30 +918,24 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
+      <c r="F1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" s="11" customFormat="1" ht="33">
-      <c r="A2" s="41">
+    <row r="2" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.7">
+      <c r="A2" s="39">
         <v>1</v>
       </c>
       <c r="B2" s="12">
@@ -957,29 +945,25 @@
         <v>18</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="E2" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="15"/>
-      <c r="G2" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="H2" s="15" t="s">
+      <c r="G2" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I2" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="J2" s="20" t="s">
+      <c r="H2" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="I2" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="K2" s="20" t="s">
-        <v>29</v>
-      </c>
     </row>
-    <row r="3" spans="1:11" s="11" customFormat="1">
+    <row r="3" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.7">
       <c r="A3" s="21">
         <v>5</v>
       </c>
@@ -987,104 +971,92 @@
         <v>11</v>
       </c>
       <c r="C3" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="21" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" s="23" t="s">
+        <v>29</v>
+      </c>
+      <c r="F3" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="I3" s="20" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" s="11" customFormat="1" ht="49.5" x14ac:dyDescent="0.7">
+      <c r="A4" s="26">
+        <v>6</v>
+      </c>
+      <c r="B4" s="27">
+        <v>1</v>
+      </c>
+      <c r="C4" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="21" t="s">
-        <v>34</v>
-      </c>
-      <c r="E3" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="F3" s="23"/>
-      <c r="G3" s="24" t="s">
+      <c r="D4" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="E4" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>23</v>
+      </c>
+      <c r="G4" s="32" t="s">
+        <v>24</v>
+      </c>
+      <c r="H4" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" s="20" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.7">
+      <c r="A5" s="33">
+        <v>6</v>
+      </c>
+      <c r="B5" s="34">
+        <v>7</v>
+      </c>
+      <c r="C5" s="35" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="34" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" s="36" t="s">
         <v>31</v>
       </c>
-      <c r="H3" s="25" t="s">
+      <c r="F5" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="G5" s="38" t="s">
         <v>24</v>
       </c>
-      <c r="I3" s="26" t="s">
-        <v>25</v>
-      </c>
-      <c r="J3" s="20" t="s">
+      <c r="H5" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5" s="20" t="s">
         <v>27</v>
-      </c>
-      <c r="K3" s="20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" s="11" customFormat="1" ht="49.5">
-      <c r="A4" s="27">
-        <v>6</v>
-      </c>
-      <c r="B4" s="28">
-        <v>1</v>
-      </c>
-      <c r="C4" s="29" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="30" t="s">
-        <v>34</v>
-      </c>
-      <c r="E4" s="30" t="s">
-        <v>28</v>
-      </c>
-      <c r="F4" s="31"/>
-      <c r="G4" s="32" t="s">
-        <v>32</v>
-      </c>
-      <c r="H4" s="31" t="s">
-        <v>24</v>
-      </c>
-      <c r="I4" s="33" t="s">
-        <v>25</v>
-      </c>
-      <c r="J4" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="K4" s="20" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" s="11" customFormat="1">
-      <c r="A5" s="34">
-        <v>6</v>
-      </c>
-      <c r="B5" s="35">
-        <v>7</v>
-      </c>
-      <c r="C5" s="36" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" s="35" t="s">
-        <v>34</v>
-      </c>
-      <c r="E5" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="F5" s="37"/>
-      <c r="G5" s="38" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" s="39" t="s">
-        <v>24</v>
-      </c>
-      <c r="I5" s="40" t="s">
-        <v>25</v>
-      </c>
-      <c r="J5" s="20" t="s">
-        <v>27</v>
-      </c>
-      <c r="K5" s="20" t="s">
-        <v>29</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="I2" r:id="rId1" xr:uid="{02B8E7D3-488D-4F3C-BE7B-78FF11235118}"/>
-    <hyperlink ref="I4" r:id="rId2" xr:uid="{06625D06-66BD-4678-9017-82E48608966E}"/>
-    <hyperlink ref="I3" r:id="rId3" xr:uid="{63D6138B-3BE9-40B2-AEE5-85CCB9B20E45}"/>
-    <hyperlink ref="I5" r:id="rId4" xr:uid="{7A19A1F0-A4AC-4FBF-B2D1-315B08BAEEF7}"/>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{02B8E7D3-488D-4F3C-BE7B-78FF11235118}"/>
+    <hyperlink ref="G4" r:id="rId2" xr:uid="{06625D06-66BD-4678-9017-82E48608966E}"/>
+    <hyperlink ref="G3" r:id="rId3" xr:uid="{63D6138B-3BE9-40B2-AEE5-85CCB9B20E45}"/>
+    <hyperlink ref="G5" r:id="rId4" xr:uid="{7A19A1F0-A4AC-4FBF-B2D1-315B08BAEEF7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1093,9 +1065,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{204D97F9-B500-401B-B8CC-59FC4C1E19E8}">
   <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="16.5"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.7"/>
   <sheetData>
-    <row r="1" spans="1:11" s="4" customFormat="1" ht="49.5">
+    <row r="1" spans="1:11" s="4" customFormat="1" ht="49.5" x14ac:dyDescent="0.7">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1130,8 +1102,8 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" s="11" customFormat="1" ht="49.5">
-      <c r="A2" s="42" t="s">
+    <row r="2" spans="1:11" s="11" customFormat="1" ht="49.5" x14ac:dyDescent="0.7">
+      <c r="A2" s="40" t="s">
         <v>11</v>
       </c>
       <c r="B2" s="5">
@@ -1158,7 +1130,7 @@
         <v>17</v>
       </c>
       <c r="K2" s="20" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>